<commit_message>
maintenance synchronization after lab meeting prestation and updates
</commit_message>
<xml_diff>
--- a/data/Nutrients/volcano.xlsx
+++ b/data/Nutrients/volcano.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/keanurochette/Desktop/Git Hub Repository/MOBEAST/data/Nutrients/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB0CFBF-643A-4544-8425-70CE5F1BE02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED55021E-43D4-604D-AAA2-526493275541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17220" activeTab="1" xr2:uid="{EA40AD60-2F8B-204E-A3EC-D3097759E413}"/>
   </bookViews>
@@ -112,14 +112,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -1122,15 +1121,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2F5635A-50AF-EF45-BDA5-7FF6F944EF95}">
-  <dimension ref="C1:G75"/>
+  <dimension ref="C1:G30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="2" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C2" s="5"/>
@@ -1140,25 +1139,25 @@
       <c r="G2" s="5"/>
     </row>
     <row r="3" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
     </row>
     <row r="6" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C6" s="5"/>
@@ -1168,25 +1167,25 @@
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
     </row>
     <row r="8" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="9" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="10" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C10" s="5"/>
@@ -1203,18 +1202,18 @@
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
     </row>
     <row r="13" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C14" s="5"/>
@@ -1224,25 +1223,25 @@
       <c r="G14" s="5"/>
     </row>
     <row r="15" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
     </row>
     <row r="16" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C18" s="5"/>
@@ -1259,18 +1258,18 @@
       <c r="G19" s="5"/>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
     </row>
     <row r="22" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C22" s="5"/>
@@ -1287,18 +1286,18 @@
       <c r="G23" s="5"/>
     </row>
     <row r="24" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="26" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C26" s="5"/>
@@ -1322,11 +1321,11 @@
       <c r="G28" s="5"/>
     </row>
     <row r="29" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
     </row>
     <row r="30" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C30" s="5"/>
@@ -1335,91 +1334,6 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-    </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-      <c r="E60" s="6"/>
-    </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C61" s="6"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
-    </row>
-    <row r="62" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C62" s="6"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="6"/>
-    </row>
-    <row r="63" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="6"/>
-    </row>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="6"/>
-    </row>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
-      <c r="E65" s="6"/>
-    </row>
-    <row r="66" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="6"/>
-    </row>
-    <row r="67" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C67" s="6"/>
-      <c r="D67" s="6"/>
-      <c r="E67" s="6"/>
-    </row>
-    <row r="68" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C68" s="6"/>
-      <c r="D68" s="6"/>
-      <c r="E68" s="6"/>
-    </row>
-    <row r="69" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C69" s="6"/>
-      <c r="D69" s="6"/>
-      <c r="E69" s="6"/>
-    </row>
-    <row r="70" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C70" s="6"/>
-      <c r="D70" s="6"/>
-      <c r="E70" s="6"/>
-    </row>
-    <row r="71" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C71" s="6"/>
-      <c r="D71" s="6"/>
-      <c r="E71" s="6"/>
-    </row>
-    <row r="72" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C72" s="6"/>
-      <c r="D72" s="6"/>
-      <c r="E72" s="6"/>
-    </row>
-    <row r="73" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C73" s="6"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="6"/>
-    </row>
-    <row r="74" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C74" s="6"/>
-      <c r="D74" s="6"/>
-      <c r="E74" s="6"/>
-    </row>
-    <row r="75" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C75" s="6"/>
-      <c r="D75" s="6"/>
-      <c r="E75" s="6"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>